<commit_message>
feat: full flow working - excel, reporter and email integrated
</commit_message>
<xml_diff>
--- a/output/Relatorio Consolidado - 09-05-2026.xlsx
+++ b/output/Relatorio Consolidado - 09-05-2026.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1292,6 +1292,822 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>6400</v>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>01/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>Monitor 27'</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t>02/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="F28" s="1" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>03/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Webcam HD</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>560</v>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>04/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>Marcos Teixeira</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>450</v>
+      </c>
+      <c r="F30" s="1" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t>04/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>Mouse Sem Fio</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F31" s="1" t="n">
+        <v>900</v>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H31" s="1" t="inlineStr">
+        <is>
+          <t>05/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>390</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>1170</v>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>06/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F33" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H33" s="1" t="inlineStr">
+        <is>
+          <t>07/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>Monitor 27'</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="F34" s="1" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="inlineStr">
+        <is>
+          <t>08/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>Marcos Teixeira</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="F35" s="1" t="n">
+        <v>2560</v>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>09/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>1011</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>10/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>1012</v>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>Webcam HD</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>280</v>
+      </c>
+      <c r="F37" s="1" t="n">
+        <v>1120</v>
+      </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="inlineStr">
+        <is>
+          <t>11/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>1013</v>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>Mouse Sem Fio</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F38" s="1" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>11/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>1014</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>12/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>1015</v>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>Marcos Teixeira</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>390</v>
+      </c>
+      <c r="F40" s="1" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>13/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>1016</v>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>Monitor 27'</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="F41" s="1" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>14/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>450</v>
+      </c>
+      <c r="F42" s="1" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H42" s="1" t="inlineStr">
+        <is>
+          <t>15/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F43" s="1" t="n">
+        <v>6400</v>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H43" s="1" t="inlineStr">
+        <is>
+          <t>16/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>1019</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>2240</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>17/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>1020</v>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>Marcos Teixeira</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Webcam HD</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <v>280</v>
+      </c>
+      <c r="F45" s="1" t="n">
+        <v>840</v>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H45" s="1" t="inlineStr">
+        <is>
+          <t>18/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>1021</v>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>Mouse Sem Fio</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F46" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H46" s="1" t="inlineStr">
+        <is>
+          <t>19/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>1022</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>390</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>1560</v>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>20/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>1023</v>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>Monitor 27'</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="F48" s="1" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>20/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E49" s="1" t="n">
+        <v>450</v>
+      </c>
+      <c r="F49" s="1" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>21/04/2025</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add move files to repository after processing
</commit_message>
<xml_diff>
--- a/output/Relatorio Consolidado - 09-05-2026.xlsx
+++ b/output/Relatorio Consolidado - 09-05-2026.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2108,6 +2108,822 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F50" s="1" t="n">
+        <v>6400</v>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>01/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>Monitor 27'</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="F51" s="1" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>02/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E52" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="F52" s="1" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>03/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Webcam HD</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>560</v>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>04/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>Marcos Teixeira</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E54" s="1" t="n">
+        <v>450</v>
+      </c>
+      <c r="F54" s="1" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>04/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>Mouse Sem Fio</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E55" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F55" s="1" t="n">
+        <v>900</v>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>05/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>390</v>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>1170</v>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>06/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F57" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G57" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>07/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>Monitor 27'</t>
+        </is>
+      </c>
+      <c r="D58" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="F58" s="1" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G58" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>08/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>Marcos Teixeira</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E59" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="F59" s="1" t="n">
+        <v>2560</v>
+      </c>
+      <c r="G59" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H59" s="1" t="inlineStr">
+        <is>
+          <t>09/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>1011</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>10/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>1012</v>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>Webcam HD</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E61" s="1" t="n">
+        <v>280</v>
+      </c>
+      <c r="F61" s="1" t="n">
+        <v>1120</v>
+      </c>
+      <c r="G61" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>11/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>1013</v>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>Mouse Sem Fio</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E62" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F62" s="1" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G62" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>11/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>1014</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>12/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>1015</v>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>Marcos Teixeira</t>
+        </is>
+      </c>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="D64" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E64" s="1" t="n">
+        <v>390</v>
+      </c>
+      <c r="F64" s="1" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G64" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H64" s="1" t="inlineStr">
+        <is>
+          <t>13/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>1016</v>
+      </c>
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>Monitor 27'</t>
+        </is>
+      </c>
+      <c r="D65" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="F65" s="1" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G65" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H65" s="1" t="inlineStr">
+        <is>
+          <t>14/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B66" s="1" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C66" s="1" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="D66" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E66" s="1" t="n">
+        <v>450</v>
+      </c>
+      <c r="F66" s="1" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G66" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H66" s="1" t="inlineStr">
+        <is>
+          <t>15/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="inlineStr">
+        <is>
+          <t>Notebook Dell</t>
+        </is>
+      </c>
+      <c r="D67" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" s="1" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F67" s="1" t="n">
+        <v>6400</v>
+      </c>
+      <c r="G67" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H67" s="1" t="inlineStr">
+        <is>
+          <t>16/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>1019</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>2240</v>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>17/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>1020</v>
+      </c>
+      <c r="B69" s="1" t="inlineStr">
+        <is>
+          <t>Marcos Teixeira</t>
+        </is>
+      </c>
+      <c r="C69" s="1" t="inlineStr">
+        <is>
+          <t>Webcam HD</t>
+        </is>
+      </c>
+      <c r="D69" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="1" t="n">
+        <v>280</v>
+      </c>
+      <c r="F69" s="1" t="n">
+        <v>840</v>
+      </c>
+      <c r="G69" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H69" s="1" t="inlineStr">
+        <is>
+          <t>18/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>1021</v>
+      </c>
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="C70" s="1" t="inlineStr">
+        <is>
+          <t>Mouse Sem Fio</t>
+        </is>
+      </c>
+      <c r="D70" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E70" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="F70" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G70" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H70" s="1" t="inlineStr">
+        <is>
+          <t>19/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>1022</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Headset Gamer</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>390</v>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>1560</v>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>20/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>1023</v>
+      </c>
+      <c r="B72" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Alves</t>
+        </is>
+      </c>
+      <c r="C72" s="1" t="inlineStr">
+        <is>
+          <t>Monitor 27'</t>
+        </is>
+      </c>
+      <c r="D72" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E72" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="F72" s="1" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G72" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H72" s="1" t="inlineStr">
+        <is>
+          <t>20/04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B73" s="1" t="inlineStr">
+        <is>
+          <t>Juliana Ramos</t>
+        </is>
+      </c>
+      <c r="C73" s="1" t="inlineStr">
+        <is>
+          <t>SSD 1TB</t>
+        </is>
+      </c>
+      <c r="D73" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E73" s="1" t="n">
+        <v>450</v>
+      </c>
+      <c r="F73" s="1" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G73" s="1" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H73" s="1" t="inlineStr">
+        <is>
+          <t>21/04/2025</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>